<commit_message>
graphs added to .xlsx
</commit_message>
<xml_diff>
--- a/results/summary_results.xlsx
+++ b/results/summary_results.xlsx
@@ -1,25 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://woodmackenzieltd-my.sharepoint.com/personal/i34005_woodmacad_com/Documents/CSML/nodal-gnn/results/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\luisv\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72D52055-1FF5-4BD6-BF6D-234BC1026DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73845A7D-8AFB-4CF3-A8F7-2A39EBF9D895}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6DE6DC27-2E62-4C44-BE5E-FAC9AF016EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="summary_results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">summary_results!$A$2:$A$5</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">summary_results!$B$1</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">summary_results!$B$2:$B$5</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -609,7 +604,65 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>Accuracy  of  GNN Models</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -632,7 +685,10 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -869,7 +925,8 @@
         <c:axId val="1583477599"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:min val="0.999"/>
+          <c:max val="1"/>
+          <c:min val="0.99"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -937,7 +994,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0.000" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -971,6 +1028,7 @@
         <c:crossAx val="1583469439"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="2.0000000000000005E-3"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -996,12 +1054,7 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -1031,14 +1084,72 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="102"/>
+      <c14:style val="104"/>
     </mc:Choice>
     <mc:Fallback>
-      <c:style val="2"/>
+      <c:style val="4"/>
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>F1 metric for GNN models</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -1061,7 +1172,10 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1302,15 +1416,6 @@
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
-        <c:majorGridlines>
-          <c:spPr>
-            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-        </c:majorGridlines>
         <c:title>
           <c:tx>
             <c:rich>
@@ -1366,7 +1471,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1400,6 +1505,7 @@
         <c:crossAx val="1583469439"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="0.1"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1425,12 +1531,7 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -1467,7 +1568,76 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:autoTitleDeleted val="1"/>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>Precision</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" baseline="0">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t> for GNN models</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1200">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
       <c:barChart>
@@ -1490,7 +1660,10 @@
           </c:tx>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent1"/>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
             </a:solidFill>
             <a:ln>
               <a:noFill/>
@@ -1795,7 +1968,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1829,6 +2002,7 @@
         <c:crossAx val="1583469439"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
+        <c:majorUnit val="0.1"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1854,12 +2028,505 @@
       <a:schemeClr val="bg1"/>
     </a:solidFill>
     <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-      <a:solidFill>
-        <a:schemeClr val="tx1">
-          <a:lumMod val="15000"/>
-          <a:lumOff val="85000"/>
-        </a:schemeClr>
-      </a:solidFill>
+      <a:noFill/>
+      <a:round/>
+    </a:ln>
+    <a:effectLst/>
+  </c:spPr>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr/>
+      </a:pPr>
+      <a:endParaRPr lang="en-US"/>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c16r2="http://schemas.microsoft.com/office/drawing/2015/06/chart">
+  <c:date1904 val="0"/>
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t>Recall</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" baseline="0">
+                <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+                <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              </a:rPr>
+              <a:t> for GNN models</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" sz="1200">
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:endParaRPr>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="1200" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>summary_results!$B$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Accuracy</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:schemeClr val="accent2">
+                <a:lumMod val="40000"/>
+                <a:lumOff val="60000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:numFmt formatCode="#,##0.000" sourceLinked="0"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" lIns="38100" tIns="19050" rIns="38100" bIns="19050" anchor="ctr" anchorCtr="1">
+                <a:spAutoFit/>
+              </a:bodyPr>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="75000"/>
+                        <a:lumOff val="25000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>summary_results!$A$2:$A$5</c:f>
+              <c:strCache>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>GraphSAGE</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>GAT</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>MPNN</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>ECGNN</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>summary_results!$D$2:$D$5</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="4"/>
+                <c:pt idx="0">
+                  <c:v>0.90725126499999997</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.86676646700000004</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.78150134000000004</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.84248554899999994</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-FD39-4C3A-BC79-A5199EE5885D}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+        </c:dLbls>
+        <c:gapWidth val="219"/>
+        <c:overlap val="-27"/>
+        <c:axId val="1583469439"/>
+        <c:axId val="1583477599"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="1583469439"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Algorithm</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+            <a:solidFill>
+              <a:schemeClr val="tx1">
+                <a:lumMod val="15000"/>
+                <a:lumOff val="85000"/>
+              </a:schemeClr>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1583477599"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="1583477599"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="1"/>
+          <c:min val="0.5"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:schemeClr val="tx1">
+                        <a:lumMod val="65000"/>
+                        <a:lumOff val="35000"/>
+                      </a:schemeClr>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Precision</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:overlay val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="-5400000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:schemeClr val="tx1">
+                      <a:lumMod val="65000"/>
+                      <a:lumOff val="35000"/>
+                    </a:schemeClr>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+        </c:title>
+        <c:numFmt formatCode="#,##0.0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:noFill/>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr rot="-60000000" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1">
+                    <a:lumMod val="65000"/>
+                    <a:lumOff val="35000"/>
+                  </a:schemeClr>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="1583469439"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+        <c:majorUnit val="0.1"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
+        <c16r3:dataDisplayOptions16>
+          <c16r3:dispNaAsBlank val="1"/>
+        </c16r3:dataDisplayOptions16>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:schemeClr val="bg1"/>
+    </a:solidFill>
+    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+      <a:noFill/>
       <a:round/>
     </a:ln>
     <a:effectLst/>
@@ -1923,42 +2590,8 @@
 </file>
 
 <file path=xl/charts/colors2.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
-  <a:schemeClr val="accent1"/>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinear" id="15">
   <a:schemeClr val="accent2"/>
-  <a:schemeClr val="accent3"/>
-  <a:schemeClr val="accent4"/>
-  <a:schemeClr val="accent5"/>
-  <a:schemeClr val="accent6"/>
-  <cs:variation/>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-    <a:lumOff val="20000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="80000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="60000"/>
-    <a:lumOff val="40000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-    <a:lumOff val="30000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="70000"/>
-  </cs:variation>
-  <cs:variation>
-    <a:lumMod val="50000"/>
-    <a:lumOff val="50000"/>
-  </cs:variation>
 </cs:colorStyle>
 </file>
 
@@ -2002,6 +2635,46 @@
 </cs:colorStyle>
 </file>
 
+<file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="10">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent2"/>
+  <a:schemeClr val="accent3"/>
+  <a:schemeClr val="accent4"/>
+  <a:schemeClr val="accent5"/>
+  <a:schemeClr val="accent6"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
+</cs:colorStyle>
+</file>
+
 <file path=xl/charts/style1.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
@@ -3009,6 +3682,509 @@
 </file>
 
 <file path=xl/charts/style3.xml><?xml version="1.0" encoding="utf-8"?>
+<cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
+  <cs:axisTitle>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:axisTitle>
+  <cs:categoryAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:categoryAxis>
+  <cs:chartArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="bg1"/>
+      </a:solidFill>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="1000" kern="1200"/>
+  </cs:chartArea>
+  <cs:dataLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="75000"/>
+        <a:lumOff val="25000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataLabel>
+  <cs:dataLabelCallout>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln>
+        <a:solidFill>
+          <a:schemeClr val="dk1">
+            <a:lumMod val="25000"/>
+            <a:lumOff val="75000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+    <cs:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="clip" horzOverflow="clip" vert="horz" wrap="square" lIns="36576" tIns="18288" rIns="36576" bIns="18288" anchor="ctr" anchorCtr="1">
+      <a:spAutoFit/>
+    </cs:bodyPr>
+  </cs:dataLabelCallout>
+  <cs:dataPoint>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint>
+  <cs:dataPoint3D>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:dataPoint3D>
+  <cs:dataPointLine>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="28575" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointLine>
+  <cs:dataPointMarker>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1">
+      <cs:styleClr val="auto"/>
+    </cs:fillRef>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointMarker>
+  <cs:dataPointMarkerLayout symbol="circle" size="5"/>
+  <cs:dataPointWireframe>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="1"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dataPointWireframe>
+  <cs:dataTable>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:dataTable>
+  <cs:downBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="dk1">
+          <a:lumMod val="65000"/>
+          <a:lumOff val="35000"/>
+        </a:schemeClr>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:downBar>
+  <cs:dropLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:dropLine>
+  <cs:errorBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="65000"/>
+            <a:lumOff val="35000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:errorBar>
+  <cs:floor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:floor>
+  <cs:gridlineMajor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMajor>
+  <cs:gridlineMinor>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="5000"/>
+            <a:lumOff val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:gridlineMinor>
+  <cs:hiLoLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="75000"/>
+            <a:lumOff val="25000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:hiLoLine>
+  <cs:leaderLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:leaderLine>
+  <cs:legend>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:legend>
+  <cs:plotArea mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea>
+  <cs:plotArea3D mods="allowNoFillOverride allowNoLineOverride">
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+  </cs:plotArea3D>
+  <cs:seriesAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:seriesAxis>
+  <cs:seriesLine>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="35000"/>
+            <a:lumOff val="65000"/>
+          </a:schemeClr>
+        </a:solidFill>
+        <a:round/>
+      </a:ln>
+    </cs:spPr>
+  </cs:seriesLine>
+  <cs:title>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="1400" b="0" kern="1200" spc="0" baseline="0"/>
+  </cs:title>
+  <cs:trendline>
+    <cs:lnRef idx="0">
+      <cs:styleClr val="auto"/>
+    </cs:lnRef>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:ln w="19050" cap="rnd">
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:prstDash val="sysDot"/>
+      </a:ln>
+    </cs:spPr>
+  </cs:trendline>
+  <cs:trendlineLabel>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:trendlineLabel>
+  <cs:upBar>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="dk1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:solidFill>
+        <a:schemeClr val="lt1"/>
+      </a:solidFill>
+      <a:ln w="9525">
+        <a:solidFill>
+          <a:schemeClr val="tx1">
+            <a:lumMod val="15000"/>
+            <a:lumOff val="85000"/>
+          </a:schemeClr>
+        </a:solidFill>
+      </a:ln>
+    </cs:spPr>
+  </cs:upBar>
+  <cs:valueAxis>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1">
+        <a:lumMod val="65000"/>
+        <a:lumOff val="35000"/>
+      </a:schemeClr>
+    </cs:fontRef>
+    <cs:defRPr sz="900" kern="1200"/>
+  </cs:valueAxis>
+  <cs:wall>
+    <cs:lnRef idx="0"/>
+    <cs:fillRef idx="0"/>
+    <cs:effectRef idx="0"/>
+    <cs:fontRef idx="minor">
+      <a:schemeClr val="tx1"/>
+    </cs:fontRef>
+    <cs:spPr>
+      <a:noFill/>
+      <a:ln>
+        <a:noFill/>
+      </a:ln>
+    </cs:spPr>
+  </cs:wall>
+</cs:chartStyle>
+</file>
+
+<file path=xl/charts/style4.xml><?xml version="1.0" encoding="utf-8"?>
 <cs:chartStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" id="201">
   <cs:axisTitle>
     <cs:lnRef idx="0"/>
@@ -3620,6 +4796,44 @@
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3E9E44D5-76F6-49AA-9510-BEA3009860AC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr>
+          <a:graphicFrameLocks/>
+        </xdr:cNvGraphicFramePr>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>

</xml_diff>

<commit_message>
feat importance + model baseline added
</commit_message>
<xml_diff>
--- a/results/summary_results.xlsx
+++ b/results/summary_results.xlsx
@@ -8,18 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://woodmackenzieltd-my.sharepoint.com/personal/i34005_woodmacad_com/Documents/CSML/nodal-gnn/results/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72D52055-1FF5-4BD6-BF6D-234BC1026DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{72D52055-1FF5-4BD6-BF6D-234BC1026DF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5795990-BA9F-4B80-B251-7C1A08366E8D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{6DE6DC27-2E62-4C44-BE5E-FAC9AF016EC0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{6DE6DC27-2E62-4C44-BE5E-FAC9AF016EC0}"/>
   </bookViews>
   <sheets>
     <sheet name="summary_results" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">summary_results!$A$2:$A$5</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">summary_results!$B$1</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">summary_results!$B$2:$B$5</definedName>
-  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
@@ -1579,21 +1574,21 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>summary_results!$C$2:$C$5</c:f>
+              <c:f>summary_results!$D$2:$D$5</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>0.901927908</c:v>
+                  <c:v>0.90725126499999997</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.91324920600000004</c:v>
+                  <c:v>0.86676646700000004</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.86627042600000004</c:v>
+                  <c:v>0.78150134000000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.90247677500000001</c:v>
+                  <c:v>0.84248554899999994</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>

</xml_diff>